<commit_message>
Power sector calibration round 2: pumped hydro on the 11th Plan path, RPS requirement rebased to the model's basis with biomass qualifying, lifetime-based coal/nuclear retirements added for 2039–50 (BGCL documented, lifetime switch off), KEEI grid-connection costs split into the spur-line input, and the BSCpUC year-header error fixed.
</commit_message>
<xml_diff>
--- a/InputData/elec/BGCL/BGCL BAU Gen Cap Lifetime.xlsx
+++ b/InputData/elec/BGCL/BGCL BAU Gen Cap Lifetime.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\China\Models\eps-china-igdp\InputData\elec\BGCL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\BGCL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{696E2BD1-8414-4717-B8F7-267A35D142F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D7FE96-0C57-4C46-898D-64B80D05C87D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{9D8EB1DD-5A7F-4AA9-9A9C-7214F3F103D3}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="10008" activeTab="1" xr2:uid="{9D8EB1DD-5A7F-4AA9-9A9C-7214F3F103D3}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Sources:</t>
   </si>
@@ -63,9 +63,6 @@
     <t>BGCL BAU Generation Capacity Lifetime</t>
   </si>
   <si>
-    <t>(none)</t>
-  </si>
-  <si>
     <t>hard coal</t>
   </si>
   <si>
@@ -139,6 +136,15 @@
   </si>
   <si>
     <t>BAU Generation Capacity Lifetime (years)</t>
+  </si>
+  <si>
+    <t>Partner (Korea team) proposal of 2026-09-08: nuclear 60 years (continued operation under the 11th Basic Plan), hydro and pumped hydro no fixed retirement (999), all other sources 30 years.</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>These lifetimes are INERT in the BAU: BUCLfCR (ctrl-settings) = 0, as in eps-us, because the model ADDS lifetime retirements to the BCRbQ schedule rather than reconciling them, and a uniform 30-yr rule retires units the 11th Plan keeps past 30 years. The same lifetimes are applied explicitly in BCRbQ for 2039-2050 (coal 30 yr, nuclear 60 yr) via the BCRbQ workbook's 39-50 tab; the 2021-2038 schedule follows the plan.</t>
   </si>
 </sst>
 </file>
@@ -170,10 +176,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -562,23 +569,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB950847-513A-41A4-B0A1-DEDEEAAEAB48}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -589,209 +607,210 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="B3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="B4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="B5">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="B6">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="B7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="B8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B8">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="B9">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B9">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="B10">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B10">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="B11">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B11">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="B12">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B12">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="B13">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B13">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+      <c r="B14">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B14">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+      <c r="B15">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B15">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+      <c r="B16">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B16">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+      <c r="B17">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B17">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="B18">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B18">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="B19">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B19">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="B20">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B20">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+      <c r="B21">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B21">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
+      <c r="B22">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B22">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+      <c r="B23">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B23">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+      <c r="B24">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B24">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
-        <v>26</v>
-      </c>
       <c r="B25">
         <v>30</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>